<commit_message>
feat(curriculum): implement student tracking, risk indicators, and tutoring modules
</commit_message>
<xml_diff>
--- a/AvanceAlumnos.xlsx
+++ b/AvanceAlumnos.xlsx
@@ -7,6 +7,8 @@
   </x:bookViews>
   <x:sheets>
     <x:sheet name="s22013691" sheetId="1" r:id="rId2"/>
+    <x:sheet name="s22013367" sheetId="2" r:id="rId5"/>
+    <x:sheet name="s22019834" sheetId="3" r:id="rId7"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="125725"/>
@@ -16,73 +18,112 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
+    <x:t>Matrícula:</x:t>
+  </x:si>
+  <x:si>
     <x:t>ultima</x:t>
   </x:si>
   <x:si>
+    <x:t>Nombre:</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Estadística</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Créditos Totales Aprobados:</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Materia</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Créditos</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Inscripción</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Último Examen</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Estado</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Lengua I</x:t>
+  </x:si>
+  <x:si>
+    <x:t>primera</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ordinario</x:t>
+  </x:si>
+  <x:si>
+    <x:t>aprobada</x:t>
+  </x:si>
+  <x:si>
+    <x:t>titulo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Pensamiento Crítico</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cálculo I</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Macroeconomía I</x:t>
+  </x:si>
+  <x:si>
+    <x:t>extraordinario</x:t>
+  </x:si>
+  <x:si>
+    <x:t>reprobada</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Historia Económica General</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Probabilidad</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cálculo II</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Finanzas</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Fidel Montemira Orozco</x:t>
+  </x:si>
+  <x:si>
     <x:t>segunda</x:t>
   </x:si>
   <x:si>
-    <x:t>Estadística</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Historia Económica General</x:t>
-  </x:si>
-  <x:si>
-    <x:t>extraordinario</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Cálculo II</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Cálculo I</x:t>
-  </x:si>
-  <x:si>
-    <x:t>reprobada</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Pensamiento Crítico</x:t>
-  </x:si>
-  <x:si>
-    <x:t>aprobada</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ordinario</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Inscripción</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Créditos</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Matrícula:</x:t>
-  </x:si>
-  <x:si>
-    <x:t>primera</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Finanzas</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Estado</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Último Examen</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Materia</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Fidel Montemira Orozco</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Nombre:</x:t>
-  </x:si>
-  <x:si>
     <x:t>s22013691</x:t>
   </x:si>
   <x:si>
-    <x:t>Créditos Totales Aprobados:</x:t>
+    <x:t>s22013367</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ana Paola Sanchez Gomez</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cursando</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Literacidad Digital</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Lectura y escritura de textos</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Microeconomía I</x:t>
+  </x:si>
+  <x:si>
+    <x:t>s22019834</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Jafeth Carballo Delgado</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Introducción a la Economía</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -472,143 +513,507 @@
   <x:sheetData>
     <x:row r="1" spans="1:5">
       <x:c r="A1" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5">
       <x:c r="A2" s="1" t="s">
-        <x:v>20</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>22</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>32</x:v>
+        <x:v>58</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
       <x:c r="A4" s="2" t="s">
-        <x:v>18</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>12</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C4" s="2" t="s">
-        <x:v>11</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D4" s="2" t="s">
-        <x:v>17</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E4" s="2" t="s">
-        <x:v>16</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:5">
       <x:c r="A5" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="0">
-        <x:v>6</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:5">
       <x:c r="A6" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B6" s="0">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:5">
       <x:c r="A7" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="B7" s="0">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B7" s="0">
-        <x:v>9</x:v>
-      </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:5">
       <x:c r="A8" s="0" t="s">
-        <x:v>5</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0">
-        <x:v>9</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>4</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:5">
       <x:c r="A9" s="0" t="s">
-        <x:v>3</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B9" s="0">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>7</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:5">
       <x:c r="A10" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B10" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:5">
+      <x:c r="A11" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="B11" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:5">
+      <x:c r="A12" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B12" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C12" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E12" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:5">
+      <x:c r="A13" s="0" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B13" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C13" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D13" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E13" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:5">
+      <x:c r="A14" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B14" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C14" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D14" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E14" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:E5"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="25.996339" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24.424911" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10.567768" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26.282054" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:5">
+      <x:c r="A1" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:5">
+      <x:c r="A2" s="1" t="s">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E2" s="0">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:5">
+      <x:c r="A4" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:5">
+      <x:c r="A5" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B5" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:5">
+      <x:c r="A6" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B6" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:5">
+      <x:c r="A7" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B7" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:5">
+      <x:c r="A8" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B8" s="0">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:E4"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="25.996339" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="21.853482" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10.567768" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26.282054" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:5">
+      <x:c r="A1" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:5">
+      <x:c r="A2" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E2" s="0">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:5">
+      <x:c r="A4" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B4" s="2" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C4" s="2" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="D4" s="2" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E4" s="2" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:5">
+      <x:c r="A5" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B5" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:5">
+      <x:c r="A6" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B6" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:5">
+      <x:c r="A7" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B7" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:5">
+      <x:c r="A8" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B8" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:5">
+      <x:c r="A9" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B9" s="0">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:5">
+      <x:c r="A10" s="0" t="s">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="B10" s="0">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>1</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>0</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>29</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat(curriculum):  reportes globales y exportación Word
</commit_message>
<xml_diff>
--- a/AvanceAlumnos.xlsx
+++ b/AvanceAlumnos.xlsx
@@ -9,6 +9,7 @@
     <x:sheet name="s22013691" sheetId="1" r:id="rId2"/>
     <x:sheet name="s22013367" sheetId="2" r:id="rId5"/>
     <x:sheet name="s22019834" sheetId="3" r:id="rId7"/>
+    <x:sheet name="s2231343536" sheetId="4" r:id="rId8"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="125725"/>
@@ -21,109 +22,175 @@
     <x:t>Matrícula:</x:t>
   </x:si>
   <x:si>
+    <x:t>s22013691</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TUTORÍAS REGISTRADAS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nombre:</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Fidel Montemira Orozco</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sesión 1</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>pendiente</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Créditos Totales Aprobados:</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sesión 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sesión 3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Materia</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Créditos</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Inscripción</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Último Examen</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Estado</x:t>
+  </x:si>
+  <x:si>
+    <x:t>En Riesgo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>En Rezago</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Lengua I</x:t>
+  </x:si>
+  <x:si>
+    <x:t>primera</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ordinario</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ninguno</x:t>
+  </x:si>
+  <x:si>
+    <x:t>False</x:t>
+  </x:si>
+  <x:si>
+    <x:t>True</x:t>
+  </x:si>
+  <x:si>
+    <x:t>toma de decisiones</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cursando</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cálculo I</x:t>
+  </x:si>
+  <x:si>
+    <x:t>aprobada</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cálculo II</x:t>
+  </x:si>
+  <x:si>
+    <x:t>extraordinario</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Probabilidad</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Macroeconomía I</x:t>
+  </x:si>
+  <x:si>
+    <x:t>titulo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Estadística</x:t>
+  </x:si>
+  <x:si>
+    <x:t>segunda</x:t>
+  </x:si>
+  <x:si>
     <x:t>ultima</x:t>
   </x:si>
   <x:si>
-    <x:t>Nombre:</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Estadística</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Créditos Totales Aprobados:</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Materia</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Créditos</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Inscripción</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Último Examen</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Estado</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Lengua I</x:t>
-  </x:si>
-  <x:si>
-    <x:t>primera</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ordinario</x:t>
-  </x:si>
-  <x:si>
-    <x:t>aprobada</x:t>
-  </x:si>
-  <x:si>
-    <x:t>titulo</x:t>
+    <x:t>optativa</x:t>
+  </x:si>
+  <x:si>
+    <x:t>s22013367</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ana Paola Sanchez Gomez</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Lectura y escritura de textos académicos</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Literacidad Digital</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Microeconomía I</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Lectura y escritura de textos</x:t>
+  </x:si>
+  <x:si>
+    <x:t>s22019834</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Jafeth Carballo Delgado</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Literacidad digital</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Introducción a la Economía</x:t>
   </x:si>
   <x:si>
     <x:t>Pensamiento Crítico</x:t>
   </x:si>
   <x:si>
-    <x:t>Cálculo I</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Macroeconomía I</x:t>
-  </x:si>
-  <x:si>
-    <x:t>extraordinario</x:t>
-  </x:si>
-  <x:si>
-    <x:t>reprobada</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Historia Económica General</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Probabilidad</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Cálculo II</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Finanzas</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Fidel Montemira Orozco</x:t>
-  </x:si>
-  <x:si>
-    <x:t>segunda</x:t>
-  </x:si>
-  <x:si>
-    <x:t>s22013691</x:t>
-  </x:si>
-  <x:si>
-    <x:t>s22013367</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Ana Paola Sanchez Gomez</x:t>
-  </x:si>
-  <x:si>
-    <x:t>cursando</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Literacidad Digital</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Lectura y escritura de textos</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Microeconomía I</x:t>
-  </x:si>
-  <x:si>
-    <x:t>s22019834</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Jafeth Carballo Delgado</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Introducción a la Economía</x:t>
+    <x:t>prueba 3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>prueba 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ivan Maldonado</x:t>
+  </x:si>
+  <x:si>
+    <x:t>falto</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-09</x:t>
+  </x:si>
+  <x:si>
+    <x:t>prueba 1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>asistio</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2026-10-01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>s2231343536</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -504,220 +571,335 @@
   <x:dimension ref="A1:E7"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25.424911" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="18.282054" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="22.853482" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="10.567768" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="26.282054" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="10.282054" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.424911" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="9.996339" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22.853482" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="9.140625" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="9.996339" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="9.140625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:5">
+    <x:row r="1" spans="1:11">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:5">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H1" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:11">
       <x:c r="A2" s="1" t="s">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="E2" s="0">
-        <x:v>58</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:5">
-      <x:c r="A4" s="2" t="s">
+      <x:c r="H2" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B4" s="2" t="s">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C4" s="2" t="s">
+      <x:c r="I2" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J2" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="D4" s="2" t="s">
+      <x:c r="K2" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:11">
+      <x:c r="D3" s="1" t="s">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="E4" s="2" t="s">
+      <x:c r="E3" s="0">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
         <x:v>9</x:v>
       </x:c>
-    </x:row>
-    <x:row r="5" spans="1:5">
-      <x:c r="A5" s="0" t="s">
+      <x:c r="I3" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J3" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="K3" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:11">
+      <x:c r="H4" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="B5" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
+      <x:c r="I4" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J4" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="K4" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:11">
+      <x:c r="A5" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="D5" s="0" t="s">
+      <x:c r="B5" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="E5" s="0" t="s">
+      <x:c r="C5" s="2" t="s">
         <x:v>13</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" spans="1:5">
+      <x:c r="D5" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F5" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G5" s="2" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:11">
       <x:c r="A6" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B6" s="0">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:5">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:11">
       <x:c r="A7" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B7" s="0">
         <x:v>6</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:5">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:11">
       <x:c r="A8" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B8" s="0">
-        <x:v>4</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:5">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G8" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:11">
       <x:c r="A9" s="0" t="s">
-        <x:v>16</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B9" s="0">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:5">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:11">
       <x:c r="A10" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B10" s="0">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" spans="1:5">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F10" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G10" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:11">
       <x:c r="A11" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B11" s="0">
-        <x:v>8</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" spans="1:5">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F11" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G11" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" spans="1:11">
       <x:c r="A12" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B12" s="0">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="D12" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="E12" s="0" t="s">
-        <x:v>19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" spans="1:5">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F12" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G12" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:11">
       <x:c r="A13" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B13" s="0">
-        <x:v>10</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" spans="1:5">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F13" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G13" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:11">
       <x:c r="A14" s="0" t="s">
-        <x:v>3</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B14" s="0">
-        <x:v>8</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D14" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E14" s="0" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="D14" s="0" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E14" s="0" t="s">
-        <x:v>13</x:v>
+      <x:c r="F14" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G14" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:11">
+      <x:c r="A15" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B15" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C15" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="D15" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E15" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F15" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G15" s="0" t="s">
+        <x:v>22</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -737,118 +919,173 @@
   <x:dimension ref="A1:E5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25.996339" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="36.996339" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="24.424911" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="10.567768" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="26.282054" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.424911" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="9.996339" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:5">
+    <x:row r="1" spans="1:7">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>27</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:5">
+        <x:v>37</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:7">
       <x:c r="A2" s="1" t="s">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>10</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" spans="1:5">
+    <x:row r="4" spans="1:7">
       <x:c r="A4" s="2" t="s">
-        <x:v>5</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C4" s="2" t="s">
-        <x:v>7</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D4" s="2" t="s">
-        <x:v>8</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E4" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:5">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G4" s="2" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:7">
       <x:c r="A5" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B5" s="0">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:5">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:7">
       <x:c r="A6" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B6" s="0">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:7">
+      <x:c r="A7" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B7" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
         <x:v>25</x:v>
       </x:c>
-      <x:c r="D6" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E6" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:5">
-      <x:c r="A7" s="0" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B7" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="D7" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E7" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:5">
+      <x:c r="F7" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:7">
       <x:c r="A8" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B8" s="0">
         <x:v>10</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G8" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:7">
+      <x:c r="A9" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B9" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="s">
+        <x:v>22</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -873,147 +1110,355 @@
     <x:col min="3" max="3" width="10.567768" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="26.282054" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.567768" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.424911" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="9.996339" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:5">
+    <x:row r="1" spans="1:7">
       <x:c r="A1" s="1" t="s">
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>33</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:5">
+        <x:v>43</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:7">
       <x:c r="A2" s="1" t="s">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:5">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:7">
       <x:c r="A4" s="2" t="s">
-        <x:v>5</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B4" s="2" t="s">
-        <x:v>6</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C4" s="2" t="s">
-        <x:v>7</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D4" s="2" t="s">
-        <x:v>8</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E4" s="2" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:5">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F4" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G4" s="2" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:7">
       <x:c r="A5" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B5" s="0">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:5">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G5" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:7">
       <x:c r="A6" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B6" s="0">
         <x:v>4</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:7">
+      <x:c r="A7" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B7" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D7" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G7" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:7">
+      <x:c r="A8" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B8" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G8" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:7">
+      <x:c r="A9" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B9" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:7">
+      <x:c r="A10" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B10" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F10" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G10" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:7">
+      <x:c r="A11" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B11" s="0">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C11" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F11" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="G11" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:E4"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15.710625" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10.567768" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="26.282054" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="8.424911" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.424911" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="9.996339" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22.853482" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10.424911" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="6.424911" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="8.853482" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:11">
+      <x:c r="A1" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="H1" s="1" t="s">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:11">
+      <x:c r="A2" s="1" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="I2" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="J2" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="K2" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:11">
+      <x:c r="D3" s="1" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E3" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="I3" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="J3" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="K3" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:11">
+      <x:c r="H4" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="I4" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="J4" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="K4" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:11">
+      <x:c r="A5" s="2" t="s">
         <x:v>11</x:v>
       </x:c>
+      <x:c r="B5" s="2" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C5" s="2" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D5" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E5" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F5" s="2" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="G5" s="2" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:11">
+      <x:c r="A6" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="B6" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:5">
-      <x:c r="A7" s="0" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="B7" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D7" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E7" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" spans="1:5">
-      <x:c r="A8" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="B8" s="0">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" spans="1:5">
-      <x:c r="A9" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="B9" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C9" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D9" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E9" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" spans="1:5">
-      <x:c r="A10" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B10" s="0">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C10" s="0" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="D10" s="0" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="E10" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G6" s="0" t="s">
+        <x:v>22</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: motor dinámico de AFELs y catálogo estructurado de Optativas
</commit_message>
<xml_diff>
--- a/AvanceAlumnos.xlsx
+++ b/AvanceAlumnos.xlsx
@@ -20,115 +20,115 @@
     <x:t>Matrícula:</x:t>
   </x:si>
   <x:si>
+    <x:t>Lectura y escritura de textos académicos</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Nombre:</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Literacidad digital</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Situación:</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Activo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Materia</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Periodo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Créditos</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Inscripción</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Examen</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Estado</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Riesgo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Rezago</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Periodo Tutoria</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Sesión</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Fecha</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Asistencia</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Comentarios</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Lengua I</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Agosto - Enero 2026</x:t>
+  </x:si>
+  <x:si>
+    <x:t>primera</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ordinario</x:t>
+  </x:si>
+  <x:si>
+    <x:t>aprobada</x:t>
+  </x:si>
+  <x:si>
+    <x:t>False</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>pendiente</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Fidel Montemira Orozco</x:t>
+  </x:si>
+  <x:si>
     <x:t>s22013691</x:t>
   </x:si>
   <x:si>
-    <x:t>Nombre:</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Fidel Montemira Orozco</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Situación:</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Activo</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Materia</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Periodo</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Créditos</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Inscripción</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Examen</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Estado</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Riesgo</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Rezago</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Periodo Tutoria</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Sesión</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Fecha</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Asistencia</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Comentarios</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Lengua I</x:t>
+    <x:t>Introducción a la economía</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ninguno</x:t>
+  </x:si>
+  <x:si>
+    <x:t>True</x:t>
   </x:si>
   <x:si>
     <x:t>Agosto - Enero 2027</x:t>
   </x:si>
   <x:si>
-    <x:t>primera</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ordinario</x:t>
-  </x:si>
-  <x:si>
-    <x:t>si</x:t>
-  </x:si>
-  <x:si>
-    <x:t>False</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>pendiente</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Literacidad digital</x:t>
-  </x:si>
-  <x:si>
-    <x:t>titulo</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Lectura y escritura de textos académicos</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Introducción a la economía</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ninguno</x:t>
-  </x:si>
-  <x:si>
-    <x:t>True</x:t>
-  </x:si>
-  <x:si>
     <x:t>Cálculo I</x:t>
   </x:si>
   <x:si>
-    <x:t>aprobada</x:t>
-  </x:si>
-  <x:si>
     <x:t>zS23013333</x:t>
   </x:si>
   <x:si>
     <x:t>Ana Paola Sanchez Gomez</x:t>
   </x:si>
   <x:si>
-    <x:t>Agosto - Enero 2026</x:t>
+    <x:t>Probabilidad</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cursando</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -526,7 +526,7 @@
     <x:col min="3" max="3" width="8.424911" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.567768" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.139196" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="8.424911" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="9.567768" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="6.567768" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="7.424911" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="9.140625" style="0" customWidth="1"/>
@@ -542,7 +542,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>1</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:14">
@@ -550,7 +550,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>3</x:v>
+        <x:v>27</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:14">
@@ -645,7 +645,7 @@
     </x:row>
     <x:row r="7" spans="1:14">
       <x:c r="A7" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
         <x:v>20</x:v>
@@ -657,7 +657,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
         <x:v>23</x:v>
@@ -686,7 +686,7 @@
     </x:row>
     <x:row r="8" spans="1:14">
       <x:c r="A8" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
         <x:v>20</x:v>
@@ -727,7 +727,7 @@
     </x:row>
     <x:row r="9" spans="1:14">
       <x:c r="A9" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
         <x:v>20</x:v>
@@ -742,13 +742,110 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="F9" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G9" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H9" s="0" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="G9" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="H9" s="0" t="s">
+      <x:c r="J9" s="0" t="s">
         <x:v>32</x:v>
+      </x:c>
+      <x:c r="K9" s="0">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L9" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="M9" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="N9" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:14">
+      <x:c r="A10" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C10" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F10" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="G10" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H10" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J10" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="K10" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L10" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="M10" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="N10" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:14">
+      <x:c r="A11" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C11" s="0">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F11" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G11" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H11" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="J11" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="K11" s="0">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="L11" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="M11" s="0" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="N11" s="0" t="s">
+        <x:v>25</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -768,7 +865,7 @@
   <x:dimension ref="A1:N5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="9.996339" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="25.282054" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="24.424911" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="8.424911" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.567768" style="0" customWidth="1"/>
@@ -789,7 +886,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:14">
@@ -797,7 +894,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:14">
@@ -851,13 +948,13 @@
     </x:row>
     <x:row r="6" spans="1:14">
       <x:c r="A6" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C6" s="0">
-        <x:v>4</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
         <x:v>21</x:v>
@@ -866,13 +963,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
         <x:v>24</x:v>
       </x:c>
       <x:c r="H6" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="J6" s="0" t="s">
         <x:v>20</x:v>
@@ -895,7 +992,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C7" s="0">
         <x:v>9</x:v>
@@ -907,7 +1004,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="G7" s="0" t="s">
         <x:v>24</x:v>
@@ -932,6 +1029,30 @@
       </x:c>
     </x:row>
     <x:row r="8" spans="1:14">
+      <x:c r="A8" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C8" s="0">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="G8" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H8" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
       <x:c r="J8" s="0" t="s">
         <x:v>20</x:v>
       </x:c>
@@ -950,7 +1071,7 @@
     </x:row>
     <x:row r="9" spans="1:14">
       <x:c r="J9" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="K9" s="0">
         <x:v>1</x:v>
@@ -967,7 +1088,7 @@
     </x:row>
     <x:row r="10" spans="1:14">
       <x:c r="J10" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="K10" s="0">
         <x:v>2</x:v>
@@ -984,7 +1105,7 @@
     </x:row>
     <x:row r="11" spans="1:14">
       <x:c r="J11" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="K11" s="0">
         <x:v>3</x:v>

</xml_diff>